<commit_message>
Add Google Search Console verification file
</commit_message>
<xml_diff>
--- a/public/IFSCA_Regulatory_Change_Execution_Workbook.xlsx
+++ b/public/IFSCA_Regulatory_Change_Execution_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Project Portfolio\A1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8D442E7-BB38-406F-BF73-67D9E8777C92}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D93945AF-451E-4206-B166-9A1371338E3E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01 - Requirement Register" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="308">
   <si>
     <t>Req ID</t>
   </si>
@@ -1000,6 +1000,9 @@
   </si>
   <si>
     <t>V-CIP expanded - new authentication methods and infrastructure standards</t>
+  </si>
+  <si>
+    <t>5.11 provison</t>
   </si>
 </sst>
 </file>
@@ -1683,7 +1686,7 @@
         <v>35</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>36</v>
+        <v>307</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>37</v>
@@ -1906,7 +1909,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="84.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="92.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>65</v>
       </c>
@@ -1982,7 +1985,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="84.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" ht="100.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>76</v>
       </c>
@@ -2192,7 +2195,7 @@
         <v>35</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>36</v>
+        <v>307</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>99</v>
@@ -2443,7 +2446,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="64.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="67.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>76</v>
       </c>

</xml_diff>